<commit_message>
Include parsebio index structure in index creation template.
</commit_message>
<xml_diff>
--- a/backend/fms_core/static/submission_templates/Index_creation_v3_7_0.xlsx
+++ b/backend/fms_core/static/submission_templates/Index_creation_v3_7_0.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Index Creation Template</t>
   </si>
@@ -1730,6 +1730,81 @@
       <t xml:space="preserve"> 3 prime</t>
     </r>
   </si>
+  <si>
+    <t xml:space="preserve">parsebio</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 prime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">  - AATGATACGGCGACCACCGAGATCTACACTAGATCGCTCGTCGGCAGCGTCAGATGTGTATAAGAGACAG - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[ insert ] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">- AGATCGGAAGAGCACACGTCTGAACTCCAGTCAC - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[ Index 3 prime ] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">- ATCTCGTATGCCGTCTTCTGCTTG -</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 3 prime</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1739,7 +1814,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1815,12 +1890,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1913,7 +1982,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2026,10 +2095,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2108,7 +2173,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U711"/>
-  <sheetFormatPr defaultColWidth="12.65625" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6484375" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="25.83"/>
@@ -5201,7 +5266,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9:C392" type="list">
-      <formula1>Structures!$A$2:$A$18</formula1>
+      <formula1>Structures!$A$2:$A$19</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5220,8 +5285,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H386"/>
-  <sheetFormatPr defaultColWidth="12.65625" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H1000"/>
+  <sheetFormatPr defaultColWidth="12.6484375" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="233.66"/>
@@ -5423,7 +5488,7 @@
       <c r="C17" s="25"/>
     </row>
     <row r="18" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="25" t="s">
         <v>43</v>
       </c>
       <c r="B18" s="26" t="s">
@@ -5431,9 +5496,13 @@
       </c>
       <c r="C18" s="25"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25"/>
-      <c r="B19" s="25"/>
+    <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>46</v>
+      </c>
       <c r="C19" s="25"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>